<commit_message>
fix: add correct file
</commit_message>
<xml_diff>
--- a/official input.xlsx
+++ b/official input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herna\.thumbnails\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Santiago\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB7CC2D-5290-42F1-8024-BFEDBDB2D849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8DCF4F7-29D7-412F-9DDD-30F6C99290C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6390" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Premisas" sheetId="1" r:id="rId1"/>
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="653" uniqueCount="266">
   <si>
     <t>Producto:</t>
   </si>
@@ -259,7 +259,16 @@
     <t>Porcentaje depreciación Edificios</t>
   </si>
   <si>
+    <t>Porcentaje depreciación Maquinaria y Equipo</t>
+  </si>
+  <si>
     <t>Units x hour</t>
+  </si>
+  <si>
+    <t>Porcentaje depreciación Equipo de Transporte</t>
+  </si>
+  <si>
+    <t>Porcentaje depreciación Equipo de computo</t>
   </si>
   <si>
     <t>Periodos</t>
@@ -2332,51 +2341,123 @@
       </c>
     </row>
     <row r="28" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="7"/>
-      <c r="I28" s="7"/>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
+      <c r="A28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="C28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="D28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="F28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="G28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="H28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="I28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="J28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="K28" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="L28" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="29" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="1"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
-      <c r="H29" s="7"/>
-      <c r="I29" s="7"/>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
+      <c r="A29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="C29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="D29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="E29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="F29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="G29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="H29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="I29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="J29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="K29" s="7">
+        <v>0.2</v>
+      </c>
+      <c r="L29" s="7">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="30" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="1"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
-      <c r="H30" s="7"/>
-      <c r="I30" s="7"/>
-      <c r="J30" s="7"/>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
+      <c r="A30" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="C30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="D30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="E30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="F30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="G30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="H30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="I30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="J30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="K30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
+      <c r="L30" s="7">
+        <v>8.5000000000000006E-2</v>
+      </c>
     </row>
     <row r="31" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="32" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="30" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B32" s="32">
         <v>80</v>
@@ -2384,7 +2465,7 @@
     </row>
     <row r="33" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="63" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B33" s="73">
         <v>1500000</v>
@@ -2393,7 +2474,7 @@
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="63" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B34" s="64">
         <v>0.09</v>
@@ -4757,7 +4838,7 @@
     </row>
     <row r="4" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B4" s="29">
         <f>3600/B3</f>
@@ -4797,7 +4878,7 @@
     </row>
     <row r="5" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B5" s="24">
         <v>7.5</v>
@@ -4835,7 +4916,7 @@
     </row>
     <row r="6" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B6" s="24">
         <v>2</v>
@@ -4873,7 +4954,7 @@
     </row>
     <row r="7" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B7" s="24">
         <v>1</v>
@@ -4911,7 +4992,7 @@
     </row>
     <row r="8" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B8" s="24">
         <v>5</v>
@@ -4949,7 +5030,7 @@
     </row>
     <row r="9" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B9" s="24">
         <v>4</v>
@@ -4987,7 +5068,7 @@
     </row>
     <row r="10" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="33" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B10" s="34">
         <v>12</v>
@@ -5025,7 +5106,7 @@
     </row>
     <row r="11" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B11" s="36">
         <f>B4*B5*B6*B7*B8*B9*B10</f>
@@ -5251,10 +5332,10 @@
     </row>
     <row r="20" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="21" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B20" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C20" s="21">
         <v>12</v>
@@ -5312,10 +5393,10 @@
     </row>
     <row r="21" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="21" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C21" s="21">
         <v>12</v>
@@ -5373,10 +5454,10 @@
     </row>
     <row r="22" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C22" s="21">
         <v>12</v>
@@ -5434,10 +5515,10 @@
     </row>
     <row r="23" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="21" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C23" s="21">
         <v>12</v>
@@ -5495,10 +5576,10 @@
     </row>
     <row r="24" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="21" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C24" s="21">
         <v>12</v>
@@ -5556,10 +5637,10 @@
     </row>
     <row r="25" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="21" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C25" s="21">
         <v>12</v>
@@ -5617,10 +5698,10 @@
     </row>
     <row r="26" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C26" s="21">
         <v>12</v>
@@ -5678,10 +5759,10 @@
     </row>
     <row r="27" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="21" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="C27" s="21">
         <v>12</v>
@@ -5739,10 +5820,10 @@
     </row>
     <row r="28" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="21" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C28" s="21">
         <v>12</v>
@@ -5800,10 +5881,10 @@
     </row>
     <row r="29" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="21" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C29" s="21">
         <v>12</v>
@@ -5861,10 +5942,10 @@
     </row>
     <row r="30" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C30" s="21">
         <v>12</v>
@@ -5922,10 +6003,10 @@
     </row>
     <row r="31" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="21" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C31" s="21">
         <v>12</v>
@@ -5983,10 +6064,10 @@
     </row>
     <row r="32" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="21" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="B32" s="21" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C32" s="21">
         <v>12</v>
@@ -6044,10 +6125,10 @@
     </row>
     <row r="33" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="21" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C33" s="21">
         <v>120</v>
@@ -7100,7 +7181,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7154,10 +7235,10 @@
     </row>
     <row r="4" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C4" s="10">
         <v>1</v>
@@ -7172,10 +7253,10 @@
     </row>
     <row r="5" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C5" s="10">
         <v>4</v>
@@ -7190,10 +7271,10 @@
     </row>
     <row r="6" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C6" s="10">
         <v>1</v>
@@ -7208,10 +7289,10 @@
     </row>
     <row r="7" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C7" s="10">
         <v>1</v>
@@ -7226,10 +7307,10 @@
     </row>
     <row r="8" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C8" s="10">
         <v>1</v>
@@ -7244,10 +7325,10 @@
     </row>
     <row r="9" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C9" s="10">
         <v>1</v>
@@ -7262,10 +7343,10 @@
     </row>
     <row r="10" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C10" s="10">
         <v>1</v>
@@ -7280,10 +7361,10 @@
     </row>
     <row r="11" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C11" s="10">
         <v>1</v>
@@ -7298,10 +7379,10 @@
     </row>
     <row r="12" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C12" s="10">
         <v>4</v>
@@ -7316,10 +7397,10 @@
     </row>
     <row r="13" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="10" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C13" s="10">
         <v>1</v>
@@ -7334,10 +7415,10 @@
     </row>
     <row r="14" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="10" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C14" s="10">
         <v>1</v>
@@ -7352,10 +7433,10 @@
     </row>
     <row r="15" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C15" s="10">
         <v>4</v>
@@ -7370,10 +7451,10 @@
     </row>
     <row r="16" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C16" s="10">
         <v>4</v>
@@ -7388,10 +7469,10 @@
     </row>
     <row r="17" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C17" s="10">
         <v>1</v>
@@ -7406,10 +7487,10 @@
     </row>
     <row r="18" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="10" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C18" s="10">
         <v>1</v>
@@ -7424,10 +7505,10 @@
     </row>
     <row r="19" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="10" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C19" s="10">
         <v>1</v>
@@ -7442,10 +7523,10 @@
     </row>
     <row r="20" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C20" s="10">
         <v>1</v>
@@ -7460,10 +7541,10 @@
     </row>
     <row r="21" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C21" s="10">
         <v>1</v>
@@ -7478,10 +7559,10 @@
     </row>
     <row r="22" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="10" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C22" s="10">
         <v>1</v>
@@ -8500,7 +8581,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B1" s="6">
         <v>2025</v>
@@ -8538,7 +8619,7 @@
     </row>
     <row r="2" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="37" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B2" s="38">
         <v>300000</v>
@@ -8586,7 +8667,7 @@
     </row>
     <row r="3" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="37" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B3" s="38">
         <v>70000</v>
@@ -8634,7 +8715,7 @@
     </row>
     <row r="4" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="37" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B4" s="38">
         <v>70000</v>
@@ -8682,7 +8763,7 @@
     </row>
     <row r="5" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="37" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B5" s="38">
         <v>0</v>
@@ -8730,7 +8811,7 @@
     </row>
     <row r="6" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="37" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B6" s="38">
         <v>400000</v>
@@ -8778,7 +8859,7 @@
     </row>
     <row r="7" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="37" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B7" s="38">
         <v>600000</v>
@@ -8826,7 +8907,7 @@
     </row>
     <row r="8" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="37" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B8" s="38">
         <v>600001</v>
@@ -8874,7 +8955,7 @@
     </row>
     <row r="9" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="37" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B9" s="38">
         <v>400000</v>
@@ -8922,7 +9003,7 @@
     </row>
     <row r="10" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="37" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B10" s="38">
         <v>400000</v>
@@ -9084,7 +9165,7 @@
     <row r="19" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="20" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="52" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B20" s="6">
         <v>2025</v>
@@ -9122,13 +9203,13 @@
     </row>
     <row r="21" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="66" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B21" s="66">
         <v>5800000</v>
       </c>
       <c r="C21" s="66">
-        <f t="shared" ref="C21:L23" si="16">B21</f>
+        <f t="shared" ref="C21:L24" si="16">B21</f>
         <v>5800000</v>
       </c>
       <c r="D21" s="66">
@@ -9170,7 +9251,7 @@
     </row>
     <row r="22" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="66" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B22" s="66">
         <v>112000</v>
@@ -9218,7 +9299,7 @@
     </row>
     <row r="23" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="66" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B23" s="66">
         <v>45000</v>
@@ -9284,7 +9365,7 @@
     <row r="28" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="29" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="52" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B29" s="6">
         <v>2025</v>
@@ -9322,13 +9403,13 @@
     </row>
     <row r="30" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B30" s="66">
         <v>15500</v>
       </c>
       <c r="C30" s="66">
-        <f t="shared" ref="C30:L34" si="17">B30</f>
+        <f t="shared" ref="C30:L36" si="17">B30</f>
         <v>15500</v>
       </c>
       <c r="D30" s="66">
@@ -9370,7 +9451,7 @@
     </row>
     <row r="31" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B31" s="66">
         <v>16500</v>
@@ -9418,7 +9499,7 @@
     </row>
     <row r="32" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B32" s="66">
         <v>120000</v>
@@ -9466,7 +9547,7 @@
     </row>
     <row r="33" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B33" s="66">
         <v>15400</v>
@@ -9514,7 +9595,7 @@
     </row>
     <row r="34" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B34" s="66">
         <v>13450</v>
@@ -9562,49 +9643,49 @@
     </row>
     <row r="35" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="66" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B35" s="66">
         <v>12500</v>
       </c>
       <c r="C35" s="66">
-        <f t="shared" ref="C35:L35" si="18">B35</f>
+        <f>B35</f>
         <v>12500</v>
       </c>
       <c r="D35" s="66">
-        <f t="shared" si="18"/>
+        <f>C35</f>
         <v>12500</v>
       </c>
       <c r="E35" s="66">
-        <f t="shared" si="18"/>
+        <f>D35</f>
         <v>12500</v>
       </c>
       <c r="F35" s="66">
-        <f t="shared" si="18"/>
+        <f>E35</f>
         <v>12500</v>
       </c>
       <c r="G35" s="66">
-        <f t="shared" si="18"/>
+        <f>F35</f>
         <v>12500</v>
       </c>
       <c r="H35" s="66">
-        <f t="shared" si="18"/>
+        <f>G35</f>
         <v>12500</v>
       </c>
       <c r="I35" s="66">
-        <f t="shared" si="18"/>
+        <f>H35</f>
         <v>12500</v>
       </c>
       <c r="J35" s="66">
-        <f t="shared" si="18"/>
+        <f>I35</f>
         <v>12500</v>
       </c>
       <c r="K35" s="66">
-        <f t="shared" si="18"/>
+        <f>J35</f>
         <v>12500</v>
       </c>
       <c r="L35" s="66">
-        <f t="shared" si="18"/>
+        <f>K35</f>
         <v>12500</v>
       </c>
     </row>
@@ -10597,41 +10678,41 @@
   <sheetData>
     <row r="1" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="39" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C1" s="39" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D1" s="39" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E1" s="39" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F1" s="39" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G1" s="39" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H1" s="39" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="I1" s="39" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J1" s="39" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="K1" s="39" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="L1" s="39"/>
       <c r="M1" s="39" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N1" s="39" t="s">
         <v>13</v>
@@ -10639,10 +10720,10 @@
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C2" s="42">
         <v>12000</v>
@@ -10691,10 +10772,10 @@
     </row>
     <row r="3" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="39" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C3" s="42">
         <v>10000</v>
@@ -10736,10 +10817,10 @@
     </row>
     <row r="4" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C4" s="42">
         <v>15000</v>
@@ -10780,10 +10861,10 @@
     </row>
     <row r="5" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="39" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C5" s="42">
         <v>15000</v>
@@ -10824,10 +10905,10 @@
     </row>
     <row r="6" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="39" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C6" s="42">
         <v>15000</v>
@@ -10868,10 +10949,10 @@
     </row>
     <row r="7" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="39" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C7" s="42">
         <v>16500</v>
@@ -10912,10 +10993,10 @@
     </row>
     <row r="8" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="39" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B8" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C8" s="42">
         <v>16500</v>
@@ -10956,10 +11037,10 @@
     </row>
     <row r="9" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="39" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C9" s="42">
         <v>16500</v>
@@ -11000,10 +11081,10 @@
     </row>
     <row r="10" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="39" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C10" s="42">
         <v>21000</v>
@@ -11044,10 +11125,10 @@
     </row>
     <row r="11" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="39" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C11" s="42">
         <v>21000</v>
@@ -11088,10 +11169,10 @@
     </row>
     <row r="12" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="39" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C12" s="42">
         <v>16500</v>
@@ -11132,10 +11213,10 @@
     </row>
     <row r="13" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="39" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C13" s="42">
         <v>21000</v>
@@ -11176,10 +11257,10 @@
     </row>
     <row r="14" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="39" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B14" s="39" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C14" s="42">
         <v>35000</v>
@@ -11220,10 +11301,10 @@
     </row>
     <row r="15" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="39" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C15" s="42">
         <v>21000</v>
@@ -11264,10 +11345,10 @@
     </row>
     <row r="16" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="39" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B16" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C16" s="42">
         <v>25000</v>
@@ -11308,10 +11389,10 @@
     </row>
     <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="39" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C17" s="42">
         <v>21000</v>
@@ -11352,10 +11433,10 @@
     </row>
     <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="39" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C18" s="42">
         <v>21000</v>
@@ -11396,10 +11477,10 @@
     </row>
     <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="39" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B19" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C19" s="42">
         <v>18000</v>
@@ -11440,10 +11521,10 @@
     </row>
     <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="39" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C20" s="42">
         <v>25000</v>
@@ -11484,10 +11565,10 @@
     </row>
     <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="39" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B21" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C21" s="42">
         <v>25000</v>
@@ -11528,10 +11609,10 @@
     </row>
     <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="39" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B22" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C22" s="42">
         <v>35000</v>
@@ -11572,10 +11653,10 @@
     </row>
     <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="39" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B23" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C23" s="42">
         <v>50000</v>
@@ -11616,10 +11697,10 @@
     </row>
     <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="39" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B24" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C24" s="42">
         <v>10000</v>
@@ -11660,10 +11741,10 @@
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="39" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C25" s="42">
         <v>10000</v>
@@ -11704,10 +11785,10 @@
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="39" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C26" s="53">
         <v>15000</v>
@@ -11768,57 +11849,57 @@
   <sheetData>
     <row r="1" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="40" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B1" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C1" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D1" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E1" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="F1" s="40" t="s">
+        <v>145</v>
+      </c>
+      <c r="G1" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="H1" s="41" t="s">
         <v>149</v>
       </c>
-      <c r="F1" s="40" t="s">
-        <v>142</v>
-      </c>
-      <c r="G1" s="40" t="s">
-        <v>144</v>
-      </c>
-      <c r="H1" s="41" t="s">
-        <v>146</v>
-      </c>
       <c r="I1" s="40" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="J1" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K1" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L1" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M1" s="40" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="N1" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="O1" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P1" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B2" s="44"/>
       <c r="C2" s="45">
@@ -11828,7 +11909,7 @@
         <v>1</v>
       </c>
       <c r="E2" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F2" s="44"/>
       <c r="G2" s="45">
@@ -11838,7 +11919,7 @@
         <v>1</v>
       </c>
       <c r="I2" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J2" s="44"/>
       <c r="K2" s="45">
@@ -11848,7 +11929,7 @@
         <v>1</v>
       </c>
       <c r="M2" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N2" s="44"/>
       <c r="O2" s="45">
@@ -11860,7 +11941,7 @@
     </row>
     <row r="3" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B3" s="47">
         <v>0.03</v>
@@ -11870,7 +11951,7 @@
         <v>360</v>
       </c>
       <c r="E3" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F3" s="47">
         <v>0.03</v>
@@ -11880,7 +11961,7 @@
         <v>300</v>
       </c>
       <c r="I3" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J3" s="47">
         <v>0.03</v>
@@ -11890,7 +11971,7 @@
         <v>450</v>
       </c>
       <c r="M3" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N3" s="47">
         <v>0.03</v>
@@ -11902,7 +11983,7 @@
     </row>
     <row r="4" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B4" s="47">
         <v>0.2</v>
@@ -11912,7 +11993,7 @@
         <v>2400</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F4" s="47">
         <v>0.2</v>
@@ -11922,7 +12003,7 @@
         <v>2000</v>
       </c>
       <c r="I4" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J4" s="47">
         <v>0.2</v>
@@ -11932,7 +12013,7 @@
         <v>3000</v>
       </c>
       <c r="M4" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N4" s="47">
         <v>0.2</v>
@@ -11944,7 +12025,7 @@
     </row>
     <row r="5" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B5" s="47">
         <v>0.13</v>
@@ -11954,7 +12035,7 @@
         <v>1560</v>
       </c>
       <c r="E5" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F5" s="47">
         <v>0.13</v>
@@ -11964,7 +12045,7 @@
         <v>1300</v>
       </c>
       <c r="I5" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J5" s="47">
         <v>0.13</v>
@@ -11974,7 +12055,7 @@
         <v>1950</v>
       </c>
       <c r="M5" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N5" s="47">
         <v>0.13</v>
@@ -11986,29 +12067,29 @@
     </row>
     <row r="6" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B6" s="44"/>
       <c r="C6" s="49"/>
       <c r="E6" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F6" s="44"/>
       <c r="G6" s="49"/>
       <c r="I6" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J6" s="44"/>
       <c r="K6" s="49"/>
       <c r="M6" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N6" s="44"/>
       <c r="O6" s="49"/>
     </row>
     <row r="7" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B7" s="44">
         <v>0.28846100000000002</v>
@@ -12018,7 +12099,7 @@
         <v>115.38440000000001</v>
       </c>
       <c r="E7" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F7" s="44">
         <v>0.28846100000000002</v>
@@ -12028,7 +12109,7 @@
         <v>96.153666666666666</v>
       </c>
       <c r="I7" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J7" s="44">
         <v>0.28846100000000002</v>
@@ -12038,7 +12119,7 @@
         <v>144.23050000000001</v>
       </c>
       <c r="M7" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N7" s="44">
         <v>0.28846100000000002</v>
@@ -12050,7 +12131,7 @@
     </row>
     <row r="8" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B8" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12060,7 +12141,7 @@
         <v>840.00000000000011</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F8" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12070,7 +12151,7 @@
         <v>700.00000000000011</v>
       </c>
       <c r="I8" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J8" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12080,7 +12161,7 @@
         <v>1050</v>
       </c>
       <c r="M8" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N8" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12092,7 +12173,7 @@
     </row>
     <row r="9" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B9" s="47">
         <v>0.02</v>
@@ -12102,7 +12183,7 @@
         <v>240</v>
       </c>
       <c r="E9" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F9" s="47">
         <v>0.02</v>
@@ -12112,7 +12193,7 @@
         <v>200</v>
       </c>
       <c r="I9" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J9" s="47">
         <v>0.02</v>
@@ -12122,7 +12203,7 @@
         <v>300</v>
       </c>
       <c r="M9" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N9" s="47">
         <v>0.02</v>
@@ -12134,7 +12215,7 @@
     </row>
     <row r="10" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B10" s="47">
         <v>0.16</v>
@@ -12144,7 +12225,7 @@
         <v>1920</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F10" s="47">
         <v>0.10879999999999999</v>
@@ -12154,7 +12235,7 @@
         <v>1088</v>
       </c>
       <c r="I10" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J10" s="47">
         <v>0.1792</v>
@@ -12164,7 +12245,7 @@
         <v>2688</v>
       </c>
       <c r="M10" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N10" s="47">
         <v>0.1792</v>
@@ -12202,7 +12283,7 @@
     </row>
     <row r="12" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B12" s="35"/>
       <c r="C12" s="49">
@@ -12210,7 +12291,7 @@
         <v>17515.384399999999</v>
       </c>
       <c r="E12" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F12" s="35"/>
       <c r="G12" s="49">
@@ -12218,7 +12299,7 @@
         <v>14596.153666666667</v>
       </c>
       <c r="I12" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J12" s="35"/>
       <c r="K12" s="49">
@@ -12226,7 +12307,7 @@
         <v>21894.230499999998</v>
       </c>
       <c r="M12" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N12" s="35"/>
       <c r="O12" s="49">
@@ -12244,57 +12325,57 @@
     </row>
     <row r="15" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="40" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D15" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F15" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H15" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I15" s="40" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="J15" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K15" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L15" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M15" s="40" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="N15" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="O15" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P15" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B16" s="44"/>
       <c r="C16" s="45">
@@ -12304,7 +12385,7 @@
         <v>1</v>
       </c>
       <c r="E16" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F16" s="44"/>
       <c r="G16" s="45">
@@ -12314,7 +12395,7 @@
         <v>1</v>
       </c>
       <c r="I16" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J16" s="44"/>
       <c r="K16" s="45">
@@ -12324,7 +12405,7 @@
         <v>1</v>
       </c>
       <c r="M16" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N16" s="44"/>
       <c r="O16" s="45">
@@ -12336,7 +12417,7 @@
     </row>
     <row r="17" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B17" s="47">
         <v>0.03</v>
@@ -12346,7 +12427,7 @@
         <v>450</v>
       </c>
       <c r="E17" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F17" s="47">
         <v>0.03</v>
@@ -12356,7 +12437,7 @@
         <v>495</v>
       </c>
       <c r="I17" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J17" s="47">
         <v>0.03</v>
@@ -12366,7 +12447,7 @@
         <v>495</v>
       </c>
       <c r="M17" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N17" s="47">
         <v>0.03</v>
@@ -12378,7 +12459,7 @@
     </row>
     <row r="18" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B18" s="47">
         <v>0.2</v>
@@ -12388,7 +12469,7 @@
         <v>3000</v>
       </c>
       <c r="E18" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F18" s="47">
         <v>0.2</v>
@@ -12398,7 +12479,7 @@
         <v>3300</v>
       </c>
       <c r="I18" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J18" s="47">
         <v>0.2</v>
@@ -12408,7 +12489,7 @@
         <v>3300</v>
       </c>
       <c r="M18" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N18" s="47">
         <v>0.2</v>
@@ -12420,7 +12501,7 @@
     </row>
     <row r="19" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B19" s="47">
         <v>0.13</v>
@@ -12430,7 +12511,7 @@
         <v>1950</v>
       </c>
       <c r="E19" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F19" s="47">
         <v>0.13</v>
@@ -12440,7 +12521,7 @@
         <v>2145</v>
       </c>
       <c r="I19" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J19" s="47">
         <v>0.13</v>
@@ -12450,7 +12531,7 @@
         <v>2145</v>
       </c>
       <c r="M19" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N19" s="47">
         <v>0.13</v>
@@ -12462,29 +12543,29 @@
     </row>
     <row r="20" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B20" s="44"/>
       <c r="C20" s="49"/>
       <c r="E20" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="49"/>
       <c r="I20" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J20" s="44"/>
       <c r="K20" s="49"/>
       <c r="M20" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N20" s="44"/>
       <c r="O20" s="49"/>
     </row>
     <row r="21" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B21" s="44">
         <v>0.28846100000000002</v>
@@ -12494,7 +12575,7 @@
         <v>144.23050000000001</v>
       </c>
       <c r="E21" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F21" s="44">
         <v>0.28846100000000002</v>
@@ -12504,7 +12585,7 @@
         <v>158.65355000000002</v>
       </c>
       <c r="I21" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J21" s="44">
         <v>0.28846100000000002</v>
@@ -12514,7 +12595,7 @@
         <v>158.65355000000002</v>
       </c>
       <c r="M21" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N21" s="44">
         <v>0.28846100000000002</v>
@@ -12526,7 +12607,7 @@
     </row>
     <row r="22" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B22" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12536,7 +12617,7 @@
         <v>1050</v>
       </c>
       <c r="E22" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F22" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12546,7 +12627,7 @@
         <v>1155</v>
       </c>
       <c r="I22" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J22" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12556,7 +12637,7 @@
         <v>1155</v>
       </c>
       <c r="M22" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N22" s="47">
         <v>7.0000000000000007E-2</v>
@@ -12568,7 +12649,7 @@
     </row>
     <row r="23" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B23" s="47">
         <v>0.02</v>
@@ -12578,7 +12659,7 @@
         <v>300</v>
       </c>
       <c r="E23" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F23" s="47">
         <v>0.02</v>
@@ -12588,7 +12669,7 @@
         <v>330</v>
       </c>
       <c r="I23" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J23" s="47">
         <v>0.02</v>
@@ -12598,7 +12679,7 @@
         <v>330</v>
       </c>
       <c r="M23" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N23" s="47">
         <v>0.02</v>
@@ -12610,14 +12691,14 @@
     </row>
     <row r="24" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B24" s="47">
         <v>0.1792</v>
       </c>
       <c r="C24" s="49"/>
       <c r="E24" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F24" s="47">
         <v>0.21360000000000001</v>
@@ -12627,7 +12708,7 @@
         <v>3524.4</v>
       </c>
       <c r="I24" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J24" s="47">
         <v>0.21360000000000001</v>
@@ -12637,7 +12718,7 @@
         <v>3524.4</v>
       </c>
       <c r="M24" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N24" s="47">
         <v>0.21360000000000001</v>
@@ -12675,7 +12756,7 @@
     </row>
     <row r="26" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B26" s="35"/>
       <c r="C26" s="49">
@@ -12683,7 +12764,7 @@
         <v>21894.230499999998</v>
       </c>
       <c r="E26" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F26" s="35"/>
       <c r="G26" s="49">
@@ -12691,7 +12772,7 @@
         <v>24083.653549999999</v>
       </c>
       <c r="I26" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J26" s="35"/>
       <c r="K26" s="49">
@@ -12699,7 +12780,7 @@
         <v>24083.653549999999</v>
       </c>
       <c r="M26" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N26" s="35"/>
       <c r="O26" s="49">
@@ -12715,57 +12796,57 @@
     </row>
     <row r="29" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="40" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B29" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C29" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D29" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F29" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G29" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H29" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I29" s="40" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="J29" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K29" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L29" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M29" s="40" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="N29" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="O29" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P29" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B30" s="44"/>
       <c r="C30" s="45">
@@ -12775,7 +12856,7 @@
         <v>1</v>
       </c>
       <c r="E30" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F30" s="44"/>
       <c r="G30" s="45">
@@ -12785,7 +12866,7 @@
         <v>1</v>
       </c>
       <c r="I30" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J30" s="44"/>
       <c r="K30" s="45">
@@ -12795,7 +12876,7 @@
         <v>1</v>
       </c>
       <c r="M30" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N30" s="44"/>
       <c r="O30" s="45">
@@ -12807,7 +12888,7 @@
     </row>
     <row r="31" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B31" s="47">
         <v>0.03</v>
@@ -12817,7 +12898,7 @@
         <v>630</v>
       </c>
       <c r="E31" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F31" s="47">
         <v>0.03</v>
@@ -12827,7 +12908,7 @@
         <v>630</v>
       </c>
       <c r="I31" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J31" s="47">
         <v>0.03</v>
@@ -12837,7 +12918,7 @@
         <v>495</v>
       </c>
       <c r="M31" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N31" s="47">
         <v>0.03</v>
@@ -12849,7 +12930,7 @@
     </row>
     <row r="32" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B32" s="47">
         <v>0.2</v>
@@ -12859,7 +12940,7 @@
         <v>4200</v>
       </c>
       <c r="E32" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F32" s="47">
         <v>0.2</v>
@@ -12869,7 +12950,7 @@
         <v>4200</v>
       </c>
       <c r="I32" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J32" s="47">
         <v>0.2</v>
@@ -12879,7 +12960,7 @@
         <v>3300</v>
       </c>
       <c r="M32" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N32" s="47">
         <v>0.2</v>
@@ -12891,7 +12972,7 @@
     </row>
     <row r="33" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B33" s="47">
         <v>0.13</v>
@@ -12901,7 +12982,7 @@
         <v>2730</v>
       </c>
       <c r="E33" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F33" s="47">
         <v>0.13</v>
@@ -12911,7 +12992,7 @@
         <v>2730</v>
       </c>
       <c r="I33" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J33" s="47">
         <v>0.13</v>
@@ -12921,7 +13002,7 @@
         <v>2145</v>
       </c>
       <c r="M33" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N33" s="47">
         <v>0.13</v>
@@ -12933,29 +13014,29 @@
     </row>
     <row r="34" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B34" s="44"/>
       <c r="C34" s="49"/>
       <c r="E34" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F34" s="44"/>
       <c r="G34" s="49"/>
       <c r="I34" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J34" s="44"/>
       <c r="K34" s="49"/>
       <c r="M34" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N34" s="44"/>
       <c r="O34" s="49"/>
     </row>
     <row r="35" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B35" s="44">
         <v>0.28846100000000002</v>
@@ -12965,7 +13046,7 @@
         <v>201.92270000000002</v>
       </c>
       <c r="E35" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F35" s="44">
         <v>0.28846100000000002</v>
@@ -12975,7 +13056,7 @@
         <v>201.92270000000002</v>
       </c>
       <c r="I35" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J35" s="44">
         <v>0.28846100000000002</v>
@@ -12985,7 +13066,7 @@
         <v>158.65355000000002</v>
       </c>
       <c r="M35" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N35" s="44">
         <v>0.28846100000000002</v>
@@ -12997,7 +13078,7 @@
     </row>
     <row r="36" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B36" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13007,7 +13088,7 @@
         <v>1470.0000000000002</v>
       </c>
       <c r="E36" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F36" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13017,7 +13098,7 @@
         <v>1470.0000000000002</v>
       </c>
       <c r="I36" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J36" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13027,7 +13108,7 @@
         <v>1155</v>
       </c>
       <c r="M36" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N36" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13039,7 +13120,7 @@
     </row>
     <row r="37" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B37" s="47">
         <v>0.02</v>
@@ -13049,7 +13130,7 @@
         <v>420</v>
       </c>
       <c r="E37" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F37" s="47">
         <v>0.02</v>
@@ -13059,7 +13140,7 @@
         <v>420</v>
       </c>
       <c r="I37" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J37" s="47">
         <v>0.02</v>
@@ -13069,7 +13150,7 @@
         <v>330</v>
       </c>
       <c r="M37" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N37" s="47">
         <v>0.02</v>
@@ -13081,7 +13162,7 @@
     </row>
     <row r="38" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B38" s="47">
         <v>0.21360000000000001</v>
@@ -13091,7 +13172,7 @@
         <v>4485.6000000000004</v>
       </c>
       <c r="E38" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F38" s="47">
         <v>0.21360000000000001</v>
@@ -13101,7 +13182,7 @@
         <v>4485.6000000000004</v>
       </c>
       <c r="I38" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J38" s="47">
         <v>0.21360000000000001</v>
@@ -13111,7 +13192,7 @@
         <v>3524.4</v>
       </c>
       <c r="M38" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N38" s="47">
         <v>0.21360000000000001</v>
@@ -13149,7 +13230,7 @@
     </row>
     <row r="40" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B40" s="35"/>
       <c r="C40" s="49">
@@ -13157,7 +13238,7 @@
         <v>30651.922700000003</v>
       </c>
       <c r="E40" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F40" s="35"/>
       <c r="G40" s="49">
@@ -13165,7 +13246,7 @@
         <v>30651.922700000003</v>
       </c>
       <c r="I40" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J40" s="35"/>
       <c r="K40" s="49">
@@ -13173,7 +13254,7 @@
         <v>24083.653549999999</v>
       </c>
       <c r="M40" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N40" s="35"/>
       <c r="O40" s="49">
@@ -13185,21 +13266,21 @@
     <row r="42" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="43" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="40" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B43" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C43" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D43" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="44" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B44" s="44"/>
       <c r="C44" s="45">
@@ -13211,7 +13292,7 @@
     </row>
     <row r="45" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B45" s="47">
         <v>0.03</v>
@@ -13223,7 +13304,7 @@
     </row>
     <row r="46" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B46" s="47">
         <v>0.2</v>
@@ -13235,7 +13316,7 @@
     </row>
     <row r="47" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B47" s="47">
         <v>0.13</v>
@@ -13247,14 +13328,14 @@
     </row>
     <row r="48" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B48" s="44"/>
       <c r="C48" s="49"/>
     </row>
     <row r="49" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B49" s="44">
         <v>0.28846100000000002</v>
@@ -13266,7 +13347,7 @@
     </row>
     <row r="50" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B50" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13278,7 +13359,7 @@
     </row>
     <row r="51" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B51" s="47">
         <v>0.02</v>
@@ -13290,7 +13371,7 @@
     </row>
     <row r="52" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B52" s="47">
         <v>0.23519999999999999</v>
@@ -13310,7 +13391,7 @@
     </row>
     <row r="54" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B54" s="35"/>
       <c r="C54" s="49">
@@ -13322,63 +13403,63 @@
     <row r="56" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="57" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="58" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="59" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="40" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B59" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C59" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D59" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E59" s="40" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F59" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G59" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H59" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I59" s="40" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J59" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K59" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L59" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M59" s="40" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="N59" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="O59" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P59" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B60" s="44"/>
       <c r="C60" s="45">
@@ -13388,7 +13469,7 @@
         <v>1</v>
       </c>
       <c r="E60" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F60" s="44"/>
       <c r="G60" s="45">
@@ -13398,7 +13479,7 @@
         <v>1</v>
       </c>
       <c r="I60" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J60" s="44"/>
       <c r="K60" s="45">
@@ -13408,7 +13489,7 @@
         <v>1</v>
       </c>
       <c r="M60" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N60" s="44"/>
       <c r="O60" s="45">
@@ -13420,7 +13501,7 @@
     </row>
     <row r="61" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B61" s="47">
         <v>0.03</v>
@@ -13430,7 +13511,7 @@
         <v>630</v>
       </c>
       <c r="E61" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F61" s="47">
         <v>0.03</v>
@@ -13440,7 +13521,7 @@
         <v>750</v>
       </c>
       <c r="I61" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J61" s="47">
         <v>0.03</v>
@@ -13450,7 +13531,7 @@
         <v>630</v>
       </c>
       <c r="M61" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N61" s="47">
         <v>0.03</v>
@@ -13462,7 +13543,7 @@
     </row>
     <row r="62" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B62" s="47">
         <v>0.2</v>
@@ -13472,7 +13553,7 @@
         <v>4200</v>
       </c>
       <c r="E62" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F62" s="47">
         <v>0.2</v>
@@ -13482,7 +13563,7 @@
         <v>5000</v>
       </c>
       <c r="I62" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J62" s="47">
         <v>0.2</v>
@@ -13492,7 +13573,7 @@
         <v>4200</v>
       </c>
       <c r="M62" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N62" s="47">
         <v>0.2</v>
@@ -13504,7 +13585,7 @@
     </row>
     <row r="63" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B63" s="47">
         <v>0.13</v>
@@ -13514,7 +13595,7 @@
         <v>2730</v>
       </c>
       <c r="E63" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F63" s="47">
         <v>0.13</v>
@@ -13524,7 +13605,7 @@
         <v>3250</v>
       </c>
       <c r="I63" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J63" s="47">
         <v>0.13</v>
@@ -13534,7 +13615,7 @@
         <v>2730</v>
       </c>
       <c r="M63" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N63" s="47">
         <v>0.13</v>
@@ -13546,29 +13627,29 @@
     </row>
     <row r="64" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B64" s="44"/>
       <c r="C64" s="49"/>
       <c r="E64" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F64" s="44"/>
       <c r="G64" s="49"/>
       <c r="I64" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J64" s="44"/>
       <c r="K64" s="49"/>
       <c r="M64" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N64" s="44"/>
       <c r="O64" s="49"/>
     </row>
     <row r="65" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B65" s="44">
         <v>0.28846100000000002</v>
@@ -13578,7 +13659,7 @@
         <v>201.92270000000002</v>
       </c>
       <c r="E65" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F65" s="44">
         <v>0.28846100000000002</v>
@@ -13588,7 +13669,7 @@
         <v>240.38416666666669</v>
       </c>
       <c r="I65" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J65" s="44">
         <v>0.28846100000000002</v>
@@ -13598,7 +13679,7 @@
         <v>201.92270000000002</v>
       </c>
       <c r="M65" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N65" s="44">
         <v>0.28846100000000002</v>
@@ -13610,7 +13691,7 @@
     </row>
     <row r="66" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B66" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13620,7 +13701,7 @@
         <v>1470.0000000000002</v>
       </c>
       <c r="E66" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F66" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13630,7 +13711,7 @@
         <v>1750.0000000000002</v>
       </c>
       <c r="I66" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J66" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13640,7 +13721,7 @@
         <v>1470.0000000000002</v>
       </c>
       <c r="M66" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N66" s="47">
         <v>7.0000000000000007E-2</v>
@@ -13652,7 +13733,7 @@
     </row>
     <row r="67" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B67" s="47">
         <v>0.02</v>
@@ -13662,7 +13743,7 @@
         <v>420</v>
       </c>
       <c r="E67" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F67" s="47">
         <v>0.02</v>
@@ -13672,7 +13753,7 @@
         <v>500</v>
       </c>
       <c r="I67" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J67" s="47">
         <v>0.02</v>
@@ -13682,7 +13763,7 @@
         <v>420</v>
       </c>
       <c r="M67" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N67" s="47">
         <v>0.02</v>
@@ -13694,7 +13775,7 @@
     </row>
     <row r="68" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B68" s="47">
         <v>0.21360000000000001</v>
@@ -13704,7 +13785,7 @@
         <v>4485.6000000000004</v>
       </c>
       <c r="E68" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F68" s="47">
         <v>0.21360000000000001</v>
@@ -13714,7 +13795,7 @@
         <v>5340</v>
       </c>
       <c r="I68" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J68" s="47">
         <v>0.21360000000000001</v>
@@ -13724,7 +13805,7 @@
         <v>4485.6000000000004</v>
       </c>
       <c r="M68" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N68" s="47">
         <v>0.21360000000000001</v>
@@ -13762,7 +13843,7 @@
     </row>
     <row r="70" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B70" s="35"/>
       <c r="C70" s="49">
@@ -13770,7 +13851,7 @@
         <v>30651.922700000003</v>
       </c>
       <c r="E70" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F70" s="35"/>
       <c r="G70" s="49">
@@ -13778,7 +13859,7 @@
         <v>36490.38416666667</v>
       </c>
       <c r="I70" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J70" s="35"/>
       <c r="K70" s="49">
@@ -13786,7 +13867,7 @@
         <v>30651.922700000003</v>
       </c>
       <c r="M70" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N70" s="35"/>
       <c r="O70" s="49">
@@ -13798,57 +13879,57 @@
     <row r="72" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="73" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="40" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B73" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C73" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D73" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E73" s="40" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F73" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G73" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H73" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I73" s="40" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="J73" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K73" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L73" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="M73" s="40" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="N73" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="O73" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="P73" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="74" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B74" s="44"/>
       <c r="C74" s="45">
@@ -13858,7 +13939,7 @@
         <v>1</v>
       </c>
       <c r="E74" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F74" s="44"/>
       <c r="G74" s="45">
@@ -13868,7 +13949,7 @@
         <v>1</v>
       </c>
       <c r="I74" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J74" s="44"/>
       <c r="K74" s="45">
@@ -13878,7 +13959,7 @@
         <v>1</v>
       </c>
       <c r="M74" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="N74" s="44"/>
       <c r="O74" s="45">
@@ -13890,7 +13971,7 @@
     </row>
     <row r="75" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B75" s="47">
         <v>0.03</v>
@@ -13900,7 +13981,7 @@
         <v>540</v>
       </c>
       <c r="E75" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F75" s="47">
         <v>0.03</v>
@@ -13910,7 +13991,7 @@
         <v>750</v>
       </c>
       <c r="I75" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J75" s="47">
         <v>0.03</v>
@@ -13920,7 +14001,7 @@
         <v>750</v>
       </c>
       <c r="M75" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="N75" s="47">
         <v>0.03</v>
@@ -13932,7 +14013,7 @@
     </row>
     <row r="76" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B76" s="47">
         <v>0.2</v>
@@ -13942,7 +14023,7 @@
         <v>3600</v>
       </c>
       <c r="E76" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F76" s="47">
         <v>0.2</v>
@@ -13952,7 +14033,7 @@
         <v>5000</v>
       </c>
       <c r="I76" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J76" s="47">
         <v>0.2</v>
@@ -13962,7 +14043,7 @@
         <v>5000</v>
       </c>
       <c r="M76" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="N76" s="47">
         <v>0.2</v>
@@ -13974,7 +14055,7 @@
     </row>
     <row r="77" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B77" s="47">
         <v>0.13</v>
@@ -13984,7 +14065,7 @@
         <v>2340</v>
       </c>
       <c r="E77" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F77" s="47">
         <v>0.13</v>
@@ -13994,7 +14075,7 @@
         <v>3250</v>
       </c>
       <c r="I77" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J77" s="47">
         <v>0.13</v>
@@ -14004,7 +14085,7 @@
         <v>3250</v>
       </c>
       <c r="M77" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="N77" s="47">
         <v>0.13</v>
@@ -14016,29 +14097,29 @@
     </row>
     <row r="78" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B78" s="44"/>
       <c r="C78" s="49"/>
       <c r="E78" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F78" s="44"/>
       <c r="G78" s="49"/>
       <c r="I78" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J78" s="44"/>
       <c r="K78" s="49"/>
       <c r="M78" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="N78" s="44"/>
       <c r="O78" s="49"/>
     </row>
     <row r="79" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B79" s="44">
         <v>0.28846100000000002</v>
@@ -14048,7 +14129,7 @@
         <v>173.07660000000001</v>
       </c>
       <c r="E79" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F79" s="44">
         <v>0.28846100000000002</v>
@@ -14058,7 +14139,7 @@
         <v>240.38416666666669</v>
       </c>
       <c r="I79" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J79" s="44">
         <v>0.28846100000000002</v>
@@ -14068,7 +14149,7 @@
         <v>240.38416666666669</v>
       </c>
       <c r="M79" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N79" s="44">
         <v>0.28846100000000002</v>
@@ -14080,7 +14161,7 @@
     </row>
     <row r="80" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B80" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14090,7 +14171,7 @@
         <v>1260.0000000000002</v>
       </c>
       <c r="E80" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F80" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14100,7 +14181,7 @@
         <v>1750.0000000000002</v>
       </c>
       <c r="I80" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J80" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14110,7 +14191,7 @@
         <v>1750.0000000000002</v>
       </c>
       <c r="M80" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N80" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14122,7 +14203,7 @@
     </row>
     <row r="81" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B81" s="47">
         <v>0.02</v>
@@ -14132,7 +14213,7 @@
         <v>360</v>
       </c>
       <c r="E81" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F81" s="47">
         <v>0.02</v>
@@ -14142,7 +14223,7 @@
         <v>500</v>
       </c>
       <c r="I81" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J81" s="47">
         <v>0.02</v>
@@ -14152,7 +14233,7 @@
         <v>500</v>
       </c>
       <c r="M81" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="N81" s="47">
         <v>0.02</v>
@@ -14164,7 +14245,7 @@
     </row>
     <row r="82" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B82" s="47">
         <v>0.21360000000000001</v>
@@ -14174,7 +14255,7 @@
         <v>3844.8</v>
       </c>
       <c r="E82" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F82" s="47">
         <v>0.21360000000000001</v>
@@ -14184,7 +14265,7 @@
         <v>5340</v>
       </c>
       <c r="I82" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J82" s="47">
         <v>0.21360000000000001</v>
@@ -14194,7 +14275,7 @@
         <v>5340</v>
       </c>
       <c r="M82" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="N82" s="47">
         <v>0.23519999999999999</v>
@@ -14232,7 +14313,7 @@
     </row>
     <row r="84" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B84" s="35"/>
       <c r="C84" s="49">
@@ -14240,7 +14321,7 @@
         <v>26273.0766</v>
       </c>
       <c r="E84" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F84" s="35"/>
       <c r="G84" s="49">
@@ -14248,7 +14329,7 @@
         <v>36490.38416666667</v>
       </c>
       <c r="I84" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J84" s="35"/>
       <c r="K84" s="49">
@@ -14256,7 +14337,7 @@
         <v>36490.38416666667</v>
       </c>
       <c r="M84" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="N84" s="35"/>
       <c r="O84" s="49">
@@ -14268,21 +14349,21 @@
     <row r="86" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="87" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="40" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B87" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C87" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D87" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="88" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B88" s="44"/>
       <c r="C88" s="45">
@@ -14294,7 +14375,7 @@
     </row>
     <row r="89" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B89" s="47">
         <v>0.03</v>
@@ -14306,7 +14387,7 @@
     </row>
     <row r="90" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B90" s="47">
         <v>0.2</v>
@@ -14318,7 +14399,7 @@
     </row>
     <row r="91" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B91" s="47">
         <v>0.13</v>
@@ -14330,14 +14411,14 @@
     </row>
     <row r="92" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B92" s="44"/>
       <c r="C92" s="49"/>
     </row>
     <row r="93" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B93" s="44">
         <v>0.28846100000000002</v>
@@ -14349,7 +14430,7 @@
     </row>
     <row r="94" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B94" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14361,7 +14442,7 @@
     </row>
     <row r="95" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B95" s="47">
         <v>0.02</v>
@@ -14373,7 +14454,7 @@
     </row>
     <row r="96" spans="1:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B96" s="47">
         <v>0.3</v>
@@ -14393,7 +14474,7 @@
     </row>
     <row r="98" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B98" s="35"/>
       <c r="C98" s="49">
@@ -14405,45 +14486,45 @@
     <row r="100" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="101" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="40" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B101" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C101" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="D101" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E101" s="40" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F101" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G101" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H101" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="I101" s="40" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="J101" s="40" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="K101" s="40" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="L101" s="41" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
     </row>
     <row r="102" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B102" s="44"/>
       <c r="C102" s="45">
@@ -14453,7 +14534,7 @@
         <v>1</v>
       </c>
       <c r="E102" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F102" s="44"/>
       <c r="G102" s="45">
@@ -14463,7 +14544,7 @@
         <v>1</v>
       </c>
       <c r="I102" s="44" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="J102" s="44"/>
       <c r="K102" s="45">
@@ -14475,7 +14556,7 @@
     </row>
     <row r="103" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B103" s="47">
         <v>0.03</v>
@@ -14485,7 +14566,7 @@
         <v>300</v>
       </c>
       <c r="E103" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F103" s="47">
         <v>0.03</v>
@@ -14495,7 +14576,7 @@
         <v>300</v>
       </c>
       <c r="I103" s="44" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="J103" s="47">
         <v>0.03</v>
@@ -14507,7 +14588,7 @@
     </row>
     <row r="104" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B104" s="47">
         <v>0.2</v>
@@ -14517,7 +14598,7 @@
         <v>2000</v>
       </c>
       <c r="E104" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F104" s="47">
         <v>0.2</v>
@@ -14527,7 +14608,7 @@
         <v>2000</v>
       </c>
       <c r="I104" s="44" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="J104" s="47">
         <v>0.2</v>
@@ -14539,7 +14620,7 @@
     </row>
     <row r="105" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B105" s="47">
         <v>0.13</v>
@@ -14549,7 +14630,7 @@
         <v>1300</v>
       </c>
       <c r="E105" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F105" s="47">
         <v>0.13</v>
@@ -14559,7 +14640,7 @@
         <v>1300</v>
       </c>
       <c r="I105" s="44" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J105" s="47">
         <v>0.13</v>
@@ -14571,24 +14652,24 @@
     </row>
     <row r="106" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B106" s="44"/>
       <c r="C106" s="49"/>
       <c r="E106" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F106" s="44"/>
       <c r="G106" s="49"/>
       <c r="I106" s="44" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J106" s="44"/>
       <c r="K106" s="49"/>
     </row>
     <row r="107" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B107" s="44">
         <v>0.28846100000000002</v>
@@ -14598,7 +14679,7 @@
         <v>96.153666666666666</v>
       </c>
       <c r="E107" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F107" s="44">
         <v>0.28846100000000002</v>
@@ -14608,7 +14689,7 @@
         <v>96.153666666666666</v>
       </c>
       <c r="I107" s="44" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="J107" s="44">
         <v>0.28846100000000002</v>
@@ -14620,7 +14701,7 @@
     </row>
     <row r="108" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B108" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14630,7 +14711,7 @@
         <v>700.00000000000011</v>
       </c>
       <c r="E108" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F108" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14640,7 +14721,7 @@
         <v>700.00000000000011</v>
       </c>
       <c r="I108" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="J108" s="47">
         <v>7.0000000000000007E-2</v>
@@ -14652,7 +14733,7 @@
     </row>
     <row r="109" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B109" s="47">
         <v>0.02</v>
@@ -14662,7 +14743,7 @@
         <v>200</v>
       </c>
       <c r="E109" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F109" s="47">
         <v>0.02</v>
@@ -14672,7 +14753,7 @@
         <v>200</v>
       </c>
       <c r="I109" s="44" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J109" s="47">
         <v>0.02</v>
@@ -14684,7 +14765,7 @@
     </row>
     <row r="110" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B110" s="47">
         <v>0.10879999999999999</v>
@@ -14694,7 +14775,7 @@
         <v>1088</v>
       </c>
       <c r="E110" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F110" s="47">
         <v>0.10879999999999999</v>
@@ -14704,7 +14785,7 @@
         <v>1088</v>
       </c>
       <c r="I110" s="44" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="J110" s="47">
         <v>0.13</v>
@@ -14736,7 +14817,7 @@
     </row>
     <row r="112" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B112" s="35"/>
       <c r="C112" s="49">
@@ -14744,7 +14825,7 @@
         <v>14596.153666666667</v>
       </c>
       <c r="E112" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F112" s="35"/>
       <c r="G112" s="49">
@@ -14752,7 +14833,7 @@
         <v>14596.153666666667</v>
       </c>
       <c r="I112" s="35" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="J112" s="35"/>
       <c r="K112" s="49">
@@ -15669,295 +15750,295 @@
   <sheetData>
     <row r="1" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="55" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B1" s="55" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="C1" s="55" t="s">
         <v>12</v>
       </c>
       <c r="D1" s="55" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="E1" s="55" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="44" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B2" s="44" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C2" s="56" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="D2" s="57">
         <v>60000</v>
       </c>
       <c r="E2" s="56" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="44"/>
       <c r="B3" s="44" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="C3" s="56" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D3" s="57">
         <v>8000</v>
       </c>
       <c r="E3" s="56" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="44"/>
       <c r="B4" s="44" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="C4" s="56" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D4" s="57">
         <v>5000</v>
       </c>
       <c r="E4" s="56" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="44"/>
       <c r="B5" s="44" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C5" s="56" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D5" s="57">
         <v>8000</v>
       </c>
       <c r="E5" s="56" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="44" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B6" s="44" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C6" s="56" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D6" s="57">
         <v>30000</v>
       </c>
       <c r="E6" s="56" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="44"/>
       <c r="B7" s="44" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C7" s="56" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D7" s="57">
         <v>25000</v>
       </c>
       <c r="E7" s="56" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="44"/>
       <c r="B8" s="44" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C8" s="56" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="D8" s="57">
         <v>15000</v>
       </c>
       <c r="E8" s="56" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="44" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B9" s="44" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C9" s="56" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D9" s="57">
         <v>0</v>
       </c>
       <c r="E9" s="56" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="44"/>
       <c r="B10" s="44" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C10" s="56" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D10" s="57">
         <v>200000</v>
       </c>
       <c r="E10" s="56" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="44"/>
       <c r="B11" s="44" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C11" s="56" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D11" s="57">
         <v>8000</v>
       </c>
       <c r="E11" s="56" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="44"/>
       <c r="B12" s="44" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C12" s="56" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D12" s="57">
         <v>15000</v>
       </c>
       <c r="E12" s="56" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="44"/>
       <c r="B13" s="44" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="C13" s="56" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D13" s="57">
         <v>20000</v>
       </c>
       <c r="E13" s="56" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="44"/>
       <c r="B14" s="44" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="C14" s="56" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="D14" s="57">
         <v>15000</v>
       </c>
       <c r="E14" s="56" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="44"/>
       <c r="B15" s="44" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C15" s="56" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D15" s="57">
         <v>5000</v>
       </c>
       <c r="E15" s="56" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="44"/>
       <c r="B16" s="44" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C16" s="56" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D16" s="57">
         <v>10000</v>
       </c>
       <c r="E16" s="56" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="44"/>
       <c r="B17" s="44" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C17" s="56" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D17" s="57">
         <v>10000</v>
       </c>
       <c r="E17" s="56" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="44"/>
       <c r="B18" s="44" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C18" s="56" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D18" s="57">
         <v>5000</v>
       </c>
       <c r="E18" s="56" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="58"/>
       <c r="B19" s="58" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="C19" s="59" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D19" s="60">
         <v>4000</v>
       </c>
       <c r="E19" s="59" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>